<commit_message>
new run with emissions
</commit_message>
<xml_diff>
--- a/sensor_potencial_hidrico_ai/model/resultados_modelos_pca.xlsx
+++ b/sensor_potencial_hidrico_ai/model/resultados_modelos_pca.xlsx
@@ -465,34 +465,34 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.08119999999999999</v>
+        <v>0.1024</v>
       </c>
       <c r="D2" t="n">
-        <v>38.9276</v>
+        <v>40.5324</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
           <t xml:space="preserve">              precision    recall  f1-score   support
            0       0.00      0.00      0.00        99
            1       0.00      0.00      0.00       104
-           2       0.00      0.00      0.00       112
-           3       0.02      0.02      0.02        86
-           4       0.08      0.11      0.09        88
-           5       0.07      0.17      0.10        98
-           6       0.02      0.04      0.03       101
-           7       0.05      0.05      0.05        94
-           8       0.05      0.08      0.07        99
+           2       0.19      0.03      0.05       112
+           3       0.05      0.06      0.05        86
+           4       0.08      0.14      0.10        88
+           5       0.09      0.24      0.14        98
+           6       0.02      0.03      0.02       101
+           7       0.06      0.07      0.07        94
+           8       0.17      0.10      0.13        99
            9       0.00      0.00      0.00       105
-          10       0.19      0.49      0.27       121
-          11       0.04      0.02      0.03        99
-          12       0.06      0.03      0.04        94
-          13       0.10      0.11      0.11        97
+          10       0.22      0.64      0.33       121
+          11       0.12      0.02      0.03        99
+          12       0.10      0.09      0.09        94
+          13       0.10      0.13      0.12        97
           14       0.00      0.00      0.00       102
-          15       0.10      0.19      0.13        91
-          16       0.00      0.00      0.00       110
-    accuracy                           0.08      1700
-   macro avg       0.05      0.08      0.05      1700
-weighted avg       0.05      0.08      0.06      1700
+          15       0.04      0.09      0.05        91
+          16       0.03      0.01      0.01       110
+    accuracy                           0.10      1700
+   macro avg       0.08      0.10      0.07      1700
+weighted avg       0.08      0.10      0.07      1700
 </t>
         </is>
       </c>
@@ -510,34 +510,34 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.1782</v>
+        <v>0.1841</v>
       </c>
       <c r="D3" t="n">
-        <v>47.5841</v>
+        <v>47.4388</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
           <t xml:space="preserve">              precision    recall  f1-score   support
-           0       0.19      0.70      0.30        99
-           1       0.13      0.03      0.05       104
-           2       0.00      0.00      0.00       112
-           3       0.15      0.09      0.12        86
-           4       0.07      0.03      0.05        88
-           5       0.23      0.09      0.13        98
-           6       0.22      0.12      0.15       101
-           7       0.08      0.03      0.05        94
+           0       0.19      0.61      0.29        99
+           1       0.04      0.01      0.02       104
+           2       0.33      0.02      0.03       112
+           3       0.12      0.07      0.09        86
+           4       0.04      0.02      0.03        88
+           5       0.25      0.13      0.17        98
+           6       0.27      0.10      0.14       101
+           7       0.06      0.02      0.03        94
            8       0.00      0.00      0.00        99
            9       0.00      0.00      0.00       105
-          10       0.20      0.71      0.31       121
-          11       0.13      0.18      0.15        99
-          12       0.21      0.03      0.06        94
-          13       0.39      0.20      0.26        97
-          14       0.20      0.11      0.14       102
-          15       0.16      0.60      0.26        91
-          16       0.10      0.04      0.05       110
+          10       0.20      0.70      0.31       121
+          11       0.10      0.15      0.12        99
+          12       0.15      0.03      0.05        94
+          13       0.46      0.38      0.42        97
+          14       0.11      0.07      0.09       102
+          15       0.17      0.65      0.28        91
+          16       0.23      0.10      0.14       110
     accuracy                           0.18      1700
-   macro avg       0.14      0.17      0.12      1700
-weighted avg       0.14      0.18      0.12      1700
+   macro avg       0.16      0.18      0.13      1700
+weighted avg       0.16      0.18      0.13      1700
 </t>
         </is>
       </c>

</xml_diff>

<commit_message>
last results svm is better
</commit_message>
<xml_diff>
--- a/sensor_potencial_hidrico_ai/model/resultados_modelos_pca.xlsx
+++ b/sensor_potencial_hidrico_ai/model/resultados_modelos_pca.xlsx
@@ -465,34 +465,34 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.1024</v>
+        <v>0.0994</v>
       </c>
       <c r="D2" t="n">
-        <v>40.5324</v>
+        <v>37.9418</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
           <t xml:space="preserve">              precision    recall  f1-score   support
            0       0.00      0.00      0.00        99
            1       0.00      0.00      0.00       104
-           2       0.19      0.03      0.05       112
-           3       0.05      0.06      0.05        86
-           4       0.08      0.14      0.10        88
-           5       0.09      0.24      0.14        98
-           6       0.02      0.03      0.02       101
-           7       0.06      0.07      0.07        94
-           8       0.17      0.10      0.13        99
+           2       0.00      0.00      0.00       112
+           3       0.04      0.03      0.04        86
+           4       0.11      0.17      0.13        88
+           5       0.06      0.18      0.09        98
+           6       0.13      0.24      0.17       101
+           7       0.07      0.10      0.08        94
+           8       0.08      0.08      0.08        99
            9       0.00      0.00      0.00       105
-          10       0.22      0.64      0.33       121
-          11       0.12      0.02      0.03        99
-          12       0.10      0.09      0.09        94
-          13       0.10      0.13      0.12        97
+          10       0.17      0.47      0.26       121
+          11       0.06      0.01      0.02        99
+          12       0.13      0.09      0.10        94
+          13       0.15      0.16      0.16        97
           14       0.00      0.00      0.00       102
-          15       0.04      0.09      0.05        91
-          16       0.03      0.01      0.01       110
+          15       0.04      0.07      0.05        91
+          16       0.12      0.04      0.06       110
     accuracy                           0.10      1700
-   macro avg       0.08      0.10      0.07      1700
-weighted avg       0.08      0.10      0.07      1700
+   macro avg       0.07      0.10      0.07      1700
+weighted avg       0.07      0.10      0.07      1700
 </t>
         </is>
       </c>
@@ -510,34 +510,34 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.1841</v>
+        <v>0.18</v>
       </c>
       <c r="D3" t="n">
-        <v>47.4388</v>
+        <v>47.17</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
           <t xml:space="preserve">              precision    recall  f1-score   support
-           0       0.19      0.61      0.29        99
-           1       0.04      0.01      0.02       104
-           2       0.33      0.02      0.03       112
-           3       0.12      0.07      0.09        86
-           4       0.04      0.02      0.03        88
-           5       0.25      0.13      0.17        98
-           6       0.27      0.10      0.14       101
-           7       0.06      0.02      0.03        94
+           0       0.19      0.66      0.30        99
+           1       0.14      0.03      0.05       104
+           2       0.25      0.01      0.02       112
+           3       0.07      0.06      0.06        86
+           4       0.09      0.06      0.07        88
+           5       0.28      0.13      0.18        98
+           6       0.13      0.04      0.06       101
+           7       0.16      0.05      0.08        94
            8       0.00      0.00      0.00        99
            9       0.00      0.00      0.00       105
-          10       0.20      0.70      0.31       121
-          11       0.10      0.15      0.12        99
-          12       0.15      0.03      0.05        94
-          13       0.46      0.38      0.42        97
-          14       0.11      0.07      0.09       102
-          15       0.17      0.65      0.28        91
-          16       0.23      0.10      0.14       110
+          10       0.20      0.73      0.31       121
+          11       0.12      0.18      0.14        99
+          12       0.24      0.04      0.07        94
+          13       0.40      0.24      0.30        97
+          14       0.11      0.06      0.08       102
+          15       0.17      0.64      0.27        91
+          16       0.19      0.07      0.11       110
     accuracy                           0.18      1700
-   macro avg       0.16      0.18      0.13      1700
-weighted avg       0.16      0.18      0.13      1700
+   macro avg       0.16      0.18      0.12      1700
+weighted avg       0.16      0.18      0.12      1700
 </t>
         </is>
       </c>

</xml_diff>

<commit_message>
new best models and results
</commit_message>
<xml_diff>
--- a/sensor_potencial_hidrico_ai/model/resultados_modelos_pca.xlsx
+++ b/sensor_potencial_hidrico_ai/model/resultados_modelos_pca.xlsx
@@ -470,37 +470,37 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.1547</v>
+        <v>0.1529</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7072000000000001</v>
+        <v>0.7121</v>
       </c>
       <c r="E2" t="n">
-        <v>38.0424</v>
+        <v>39.7482</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
           <t xml:space="preserve">              precision    recall  f1-score   support
            0       0.00      0.00      0.00        99
-           1       0.17      0.18      0.17       104
-           2       0.14      0.08      0.10       112
-           3       0.07      0.07      0.07        86
-           4       0.09      0.15      0.11        88
-           5       0.12      0.08      0.10        98
-           6       0.24      0.22      0.23       101
-           7       0.03      0.04      0.03        94
-           8       0.13      0.11      0.12        99
+           1       0.14      0.23      0.17       104
+           2       0.16      0.11      0.13       112
+           3       0.08      0.09      0.08        86
+           4       0.11      0.12      0.12        88
+           5       0.14      0.07      0.09        98
+           6       0.14      0.14      0.14       101
+           7       0.04      0.06      0.05        94
+           8       0.17      0.13      0.15        99
            9       0.00      0.00      0.00       105
-          10       0.22      0.46      0.30       121
-          11       0.07      0.11      0.08        99
-          12       0.17      0.24      0.20        94
-          13       0.57      0.43      0.49        97
-          14       0.12      0.11      0.11       102
-          15       0.16      0.30      0.21        91
-          16       0.14      0.01      0.02       110
+          10       0.22      0.51      0.31       121
+          11       0.15      0.19      0.17        99
+          12       0.15      0.22      0.18        94
+          13       0.38      0.29      0.33        97
+          14       0.12      0.07      0.09       102
+          15       0.16      0.30      0.20        91
+          16       0.07      0.01      0.02       110
     accuracy                           0.15      1700
-   macro avg       0.14      0.15      0.14      1700
-weighted avg       0.14      0.15      0.14      1700
+   macro avg       0.13      0.15      0.13      1700
+weighted avg       0.13      0.15      0.13      1700
 </t>
         </is>
       </c>
@@ -518,37 +518,37 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.17</v>
+        <v>0.1765</v>
       </c>
       <c r="D3" t="n">
-        <v>0.7753</v>
+        <v>0.7762</v>
       </c>
       <c r="E3" t="n">
-        <v>47.6135</v>
+        <v>48.3088</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
           <t xml:space="preserve">              precision    recall  f1-score   support
-           0       0.17      0.52      0.25        99
-           1       0.00      0.00      0.00       104
-           2       0.00      0.00      0.00       112
+           0       0.18      0.61      0.28        99
+           1       0.07      0.02      0.03       104
+           2       0.50      0.01      0.02       112
            3       0.14      0.08      0.10        86
-           4       0.10      0.06      0.07        88
-           5       0.29      0.11      0.16        98
-           6       0.14      0.08      0.10       101
-           7       0.05      0.02      0.03        94
+           4       0.09      0.05      0.06        88
+           5       0.25      0.11      0.15        98
+           6       0.25      0.14      0.18       101
+           7       0.09      0.03      0.05        94
            8       0.00      0.00      0.00        99
            9       0.00      0.00      0.00       105
-          10       0.20      0.72      0.31       121
-          11       0.12      0.16      0.14        99
-          12       0.23      0.03      0.06        94
-          13       0.30      0.11      0.16        97
-          14       0.10      0.07      0.08       102
-          15       0.17      0.65      0.27        91
-          16       0.25      0.20      0.22       110
-    accuracy                           0.17      1700
-   macro avg       0.13      0.17      0.12      1700
-weighted avg       0.13      0.17      0.12      1700
+          10       0.19      0.67      0.30       121
+          11       0.10      0.16      0.13        99
+          12       0.14      0.03      0.05        94
+          13       0.44      0.28      0.34        97
+          14       0.10      0.06      0.07       102
+          15       0.17      0.64      0.27        91
+          16       0.18      0.06      0.09       110
+    accuracy                           0.18      1700
+   macro avg       0.17      0.17      0.12      1700
+weighted avg       0.17      0.18      0.13      1700
 </t>
         </is>
       </c>

</xml_diff>